<commit_message>
Auditoría SAG: pesos de riesgo de plantel tomados del informe SEPA
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/auditoria-sag/pesos-riesgo.xlsx
+++ b/auditoria-sag/pesos-riesgo.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -604,6 +604,8 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="62" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -657,6 +659,16 @@
           <t>Aplica a</t>
         </is>
       </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Borrador inicial</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Origen del peso</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -690,7 +702,7 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H2" s="5" t="n"/>
       <c r="I2" s="4" t="inlineStr">
@@ -699,6 +711,14 @@
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr"/>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -732,7 +752,7 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="H3" s="5" t="n"/>
       <c r="I3" s="4" t="inlineStr">
@@ -741,6 +761,14 @@
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -779,6 +807,14 @@
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -812,7 +848,7 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H5" s="5" t="n"/>
       <c r="I5" s="4" t="inlineStr">
@@ -821,6 +857,14 @@
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -854,7 +898,7 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H6" s="5" t="n"/>
       <c r="I6" s="4" t="inlineStr">
@@ -863,6 +907,14 @@
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -896,7 +948,7 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H7" s="5" t="n"/>
       <c r="I7" s="4" t="inlineStr">
@@ -905,6 +957,14 @@
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -943,6 +1003,14 @@
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -976,7 +1044,7 @@
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="H9" s="5" t="n"/>
       <c r="I9" s="4" t="inlineStr">
@@ -985,6 +1053,14 @@
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1027,6 +1103,14 @@
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1065,6 +1149,14 @@
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1098,7 +1190,7 @@
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="H12" s="5" t="n"/>
       <c r="I12" s="4" t="inlineStr">
@@ -1107,6 +1199,14 @@
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1140,7 +1240,7 @@
         </is>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="H13" s="5" t="n"/>
       <c r="I13" s="4" t="inlineStr">
@@ -1149,6 +1249,14 @@
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1178,7 +1286,7 @@
         </is>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="H14" s="5" t="n"/>
       <c r="I14" s="4" t="inlineStr">
@@ -1187,6 +1295,14 @@
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1229,6 +1345,14 @@
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1262,7 +1386,7 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H16" s="5" t="n"/>
       <c r="I16" s="4" t="inlineStr">
@@ -1271,6 +1395,14 @@
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1309,6 +1441,14 @@
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1338,7 +1478,7 @@
         </is>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="H18" s="5" t="n"/>
       <c r="I18" s="4" t="inlineStr">
@@ -1347,6 +1487,14 @@
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr"/>
+      <c r="K18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1389,6 +1537,14 @@
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr"/>
+      <c r="K19" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1431,6 +1587,14 @@
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1464,7 +1628,7 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H21" s="5" t="n"/>
       <c r="I21" s="4" t="inlineStr">
@@ -1473,6 +1637,14 @@
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1515,6 +1687,14 @@
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1544,7 +1724,7 @@
         </is>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="H23" s="5" t="n"/>
       <c r="I23" s="4" t="inlineStr">
@@ -1553,6 +1733,14 @@
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1586,7 +1774,7 @@
         </is>
       </c>
       <c r="G24" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H24" s="5" t="n"/>
       <c r="I24" s="4" t="inlineStr">
@@ -1595,6 +1783,14 @@
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1624,7 +1820,7 @@
         </is>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H25" s="5" t="n"/>
       <c r="I25" s="4" t="inlineStr">
@@ -1633,6 +1829,14 @@
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1662,7 +1866,7 @@
         </is>
       </c>
       <c r="G26" s="4" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="H26" s="5" t="n"/>
       <c r="I26" s="4" t="inlineStr">
@@ -1671,6 +1875,14 @@
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr"/>
+      <c r="K26" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1713,6 +1925,14 @@
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1755,6 +1975,14 @@
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1788,7 +2016,7 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H29" s="5" t="n"/>
       <c r="I29" s="4" t="inlineStr">
@@ -1797,6 +2025,14 @@
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr"/>
+      <c r="K29" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1830,7 +2066,7 @@
         </is>
       </c>
       <c r="G30" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H30" s="5" t="n"/>
       <c r="I30" s="4" t="inlineStr">
@@ -1839,6 +2075,14 @@
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr"/>
+      <c r="K30" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1885,6 +2129,14 @@
           <t>Solo ponedora</t>
         </is>
       </c>
+      <c r="K31" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1927,6 +2179,14 @@
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr"/>
+      <c r="K32" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1960,7 +2220,7 @@
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H33" s="5" t="n"/>
       <c r="I33" s="4" t="inlineStr">
@@ -1969,6 +2229,14 @@
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2007,6 +2275,14 @@
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr"/>
+      <c r="K34" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2036,7 +2312,7 @@
         </is>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H35" s="5" t="n"/>
       <c r="I35" s="4" t="inlineStr">
@@ -2045,6 +2321,14 @@
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2083,6 +2367,14 @@
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr"/>
+      <c r="K36" t="n">
+        <v>1</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2125,6 +2417,14 @@
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2167,6 +2467,14 @@
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr"/>
+      <c r="K38" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2196,7 +2504,7 @@
         </is>
       </c>
       <c r="G39" s="4" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="H39" s="5" t="n"/>
       <c r="I39" s="4" t="inlineStr">
@@ -2205,6 +2513,14 @@
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr"/>
+      <c r="K39" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2238,7 +2554,7 @@
         </is>
       </c>
       <c r="G40" s="4" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H40" s="5" t="n"/>
       <c r="I40" s="4" t="inlineStr">
@@ -2247,6 +2563,14 @@
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr"/>
+      <c r="K40" t="n">
+        <v>1</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2276,7 +2600,7 @@
         </is>
       </c>
       <c r="G41" s="4" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H41" s="5" t="n"/>
       <c r="I41" s="4" t="inlineStr">
@@ -2285,6 +2609,14 @@
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr"/>
+      <c r="K41" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2318,7 +2650,7 @@
         </is>
       </c>
       <c r="G42" s="4" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="H42" s="5" t="n"/>
       <c r="I42" s="4" t="inlineStr">
@@ -2327,6 +2659,14 @@
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr"/>
+      <c r="K42" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2360,7 +2700,7 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H43" s="5" t="n"/>
       <c r="I43" s="4" t="inlineStr">
@@ -2369,6 +2709,14 @@
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr"/>
+      <c r="K43" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -2402,7 +2750,7 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H44" s="5" t="n"/>
       <c r="I44" s="4" t="inlineStr">
@@ -2411,6 +2759,14 @@
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr"/>
+      <c r="K44" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2440,7 +2796,7 @@
         </is>
       </c>
       <c r="G45" s="4" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="H45" s="5" t="n"/>
       <c r="I45" s="4" t="inlineStr">
@@ -2449,6 +2805,14 @@
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr"/>
+      <c r="K45" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -2478,7 +2842,7 @@
         </is>
       </c>
       <c r="G46" s="4" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="H46" s="5" t="n"/>
       <c r="I46" s="4" t="inlineStr">
@@ -2487,6 +2851,14 @@
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr"/>
+      <c r="K46" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -2525,6 +2897,14 @@
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr"/>
+      <c r="K47" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -2563,6 +2943,14 @@
         </is>
       </c>
       <c r="J48" s="4" t="inlineStr"/>
+      <c r="K48" t="n">
+        <v>1</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -2601,6 +2989,14 @@
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr"/>
+      <c r="K49" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -2630,7 +3026,7 @@
         </is>
       </c>
       <c r="G50" s="4" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="H50" s="5" t="n"/>
       <c r="I50" s="4" t="inlineStr">
@@ -2643,6 +3039,14 @@
           <t>Solo ponedora</t>
         </is>
       </c>
+      <c r="K50" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -2672,7 +3076,7 @@
         </is>
       </c>
       <c r="G51" s="4" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="H51" s="5" t="n"/>
       <c r="I51" s="4" t="inlineStr">
@@ -2685,6 +3089,14 @@
           <t>Solo ponedora</t>
         </is>
       </c>
+      <c r="K51" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -2718,7 +3130,7 @@
         </is>
       </c>
       <c r="G52" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H52" s="5" t="n"/>
       <c r="I52" s="4" t="inlineStr">
@@ -2727,6 +3139,14 @@
         </is>
       </c>
       <c r="J52" s="4" t="inlineStr"/>
+      <c r="K52" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -2760,7 +3180,7 @@
         </is>
       </c>
       <c r="G53" s="4" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="H53" s="5" t="n"/>
       <c r="I53" s="4" t="inlineStr">
@@ -2769,6 +3189,14 @@
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr"/>
+      <c r="K53" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -2802,7 +3230,7 @@
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="H54" s="5" t="n"/>
       <c r="I54" s="4" t="inlineStr">
@@ -2811,6 +3239,14 @@
         </is>
       </c>
       <c r="J54" s="4" t="inlineStr"/>
+      <c r="K54" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -2853,6 +3289,14 @@
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr"/>
+      <c r="K55" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -2886,7 +3330,7 @@
         </is>
       </c>
       <c r="G56" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H56" s="5" t="n"/>
       <c r="I56" s="4" t="inlineStr">
@@ -2895,6 +3339,14 @@
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr"/>
+      <c r="K56" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -2928,7 +3380,7 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H57" s="5" t="n"/>
       <c r="I57" s="4" t="inlineStr">
@@ -2941,6 +3393,14 @@
           <t>Solo ponedora</t>
         </is>
       </c>
+      <c r="K57" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -2983,6 +3443,14 @@
           <t>No en Ponedora B</t>
         </is>
       </c>
+      <c r="K58" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -3016,7 +3484,7 @@
         </is>
       </c>
       <c r="G59" s="4" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H59" s="5" t="n"/>
       <c r="I59" s="4" t="inlineStr">
@@ -3025,6 +3493,14 @@
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr"/>
+      <c r="K59" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -3071,6 +3547,14 @@
           <t>Solo engorda</t>
         </is>
       </c>
+      <c r="K60" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -3117,6 +3601,14 @@
           <t>Solo engorda</t>
         </is>
       </c>
+      <c r="K61" t="n">
+        <v>1</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -3150,7 +3642,7 @@
         </is>
       </c>
       <c r="G62" s="4" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="H62" s="5" t="n"/>
       <c r="I62" s="4" t="inlineStr">
@@ -3163,6 +3655,14 @@
           <t>Solo engorda</t>
         </is>
       </c>
+      <c r="K62" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -3201,6 +3701,14 @@
         </is>
       </c>
       <c r="J63" s="4" t="inlineStr"/>
+      <c r="K63" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -3230,7 +3738,7 @@
         </is>
       </c>
       <c r="G64" s="4" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="H64" s="5" t="n"/>
       <c r="I64" s="4" t="inlineStr">
@@ -3239,6 +3747,14 @@
         </is>
       </c>
       <c r="J64" s="4" t="inlineStr"/>
+      <c r="K64" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -3268,7 +3784,7 @@
         </is>
       </c>
       <c r="G65" s="4" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="H65" s="5" t="n"/>
       <c r="I65" s="4" t="inlineStr">
@@ -3277,6 +3793,14 @@
         </is>
       </c>
       <c r="J65" s="4" t="inlineStr"/>
+      <c r="K65" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -3310,7 +3834,7 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H66" s="5" t="n"/>
       <c r="I66" s="4" t="inlineStr">
@@ -3319,6 +3843,14 @@
         </is>
       </c>
       <c r="J66" s="4" t="inlineStr"/>
+      <c r="K66" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -3361,6 +3893,14 @@
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr"/>
+      <c r="K67" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -3394,7 +3934,7 @@
         </is>
       </c>
       <c r="G68" s="4" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="H68" s="5" t="n"/>
       <c r="I68" s="4" t="inlineStr">
@@ -3403,6 +3943,14 @@
         </is>
       </c>
       <c r="J68" s="4" t="inlineStr"/>
+      <c r="K68" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -3436,7 +3984,7 @@
         </is>
       </c>
       <c r="G69" s="4" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="H69" s="5" t="n"/>
       <c r="I69" s="4" t="inlineStr">
@@ -3445,6 +3993,14 @@
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr"/>
+      <c r="K69" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>SEPA 2025 (criterio de Andrés)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J69"/>

</xml_diff>